<commit_message>
Let workbook dropdowns allow blanks and actually show their errors
allowBlank was off, so every unused row below the data would have been
flagged in Excel, and showErrorMessage was off, so the guidance written
into each dropdown never appeared and bad values were not blocked.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/office-hours.xlsx
+++ b/data/office-hours.xlsx
@@ -1083,7 +1083,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="C2:C400" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" error="Role must be faculty, gtf, or la." type="list">
+    <dataValidation sqref="C2:C400" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not one of the choices" error="Role must be faculty, gtf, or la." type="list">
       <formula1>"faculty,gtf,la"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2679,16 +2679,16 @@
     </row>
   </sheetData>
   <dataValidations count="4">
-    <dataValidation sqref="B2:B400" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="B2:B400" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not one of the choices" error="Office hours are Monday to Friday." type="list">
       <formula1>"Monday,Tuesday,Wednesday,Thursday,Friday"</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E400" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E2:E400" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not one of the choices" error="Use in-person or online. Blank means in-person." type="list">
       <formula1>"in-person,online"</formula1>
     </dataValidation>
-    <dataValidation sqref="H2:H400" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="H2:H400" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not one of the choices" error="Use yes or no. Blank means yes." type="list">
       <formula1>"yes,no"</formula1>
     </dataValidation>
-    <dataValidation sqref="A2:A400" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" error="Pick a name from the people sheet. Add them there first if they are new." type="list">
+    <dataValidation sqref="A2:A400" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not one of the choices" error="Pick a name from the people sheet. Add them there first if they are new." type="list">
       <formula1>PeopleNames</formula1>
     </dataValidation>
   </dataValidations>
@@ -2762,10 +2762,10 @@
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="E2:E400" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E2:E400" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not one of the choices" error="Use cancelled or added." type="list">
       <formula1>"cancelled,added"</formula1>
     </dataValidation>
-    <dataValidation sqref="A2:A400" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="A2:A400" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not one of the choices" error="Pick a name from the people sheet." type="list">
       <formula1>PeopleNames</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Count ENGR 111 coverage as ENGR 123 coverage
Everyone who helps with ENGR 111 can help with ENGR 123, so ENGR 123 was in
the site title while matching nobody in the Course filter.

Written as a rule in the settings sheet (`course_implies`) rather than as a
wider default, so it also catches anyone with an explicit courses list, and so
the next pairing is a cell edit rather than a code change. Rules chain, and a
rule that points back at itself cannot spin. ?check=1 prints what is in effect.

Also adds tools/serve.py for local previews. The stock python http.server
sends no Cache-Control at all, so a browser serves a stale assets/data.js
after an edit and you debug a change that never loaded — which is exactly what
happened while verifying this. GitHub Pages sends a real max-age, so
production was never affected.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/office-hours.xlsx
+++ b/data/office-hours.xlsx
@@ -2801,7 +2801,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2856,7 +2856,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
   </sheetData>
   <dataValidations count="2">
     <dataValidation sqref="E2:E400" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not one of the choices" error="Use cancelled or added." type="list">
@@ -2876,7 +2875,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3032,6 +3031,18 @@
       <c r="B13" s="3" t="inlineStr">
         <is>
           <t>AV C144; AV C141; Scott Engineering</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>course_implies</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>ENGR 111 -&gt; ENGR 123</t>
         </is>
       </c>
     </row>
@@ -3059,7 +3070,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -3074,7 +3084,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
@@ -3124,7 +3133,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
@@ -3132,7 +3140,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
@@ -3189,7 +3196,6 @@
         </is>
       </c>
     </row>
-    <row r="24"/>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
@@ -3218,7 +3224,6 @@
         </is>
       </c>
     </row>
-    <row r="29"/>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
@@ -3226,7 +3231,6 @@
         </is>
       </c>
     </row>
-    <row r="31"/>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Confirm AV C144 for all in-person hours; Ben is faculty
Both confirmed by the office on 25 Aug 2026.

The (AV 147) annotations still scattered through the source workbook are
stale. Nothing needed changing in the data: no shift row carries an explicit
room, so every in-person hour already resolved to default_location_* in
settings. Recorded in MIGRATION-NOTES.md so the next person to see AV 147 in
an old grid does not re-raise it.

Ben moves from gtf to faculty. His highlight and review comment are cleared in
the workbook, and the generator now keeps confirmed roles separate from
guessed ones so a re-run cannot reintroduce the guess. Ten names still await
confirmation.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/office-hours.xlsx
+++ b/data/office-hours.xlsx
@@ -162,11 +162,6 @@
     <author>migration</author>
   </authors>
   <commentList>
-    <comment ref="C5" authorId="0" shapeId="0">
-      <text>
-        <t>Guessed during the migration from the old schedules, because the grid only gave a first name or a title. Please confirm and clear the highlight. See MIGRATION-NOTES.md.</t>
-      </text>
-    </comment>
     <comment ref="C7" authorId="0" shapeId="0">
       <text>
         <t>Guessed during the migration from the old schedules, because the grid only gave a first name or a title. Please confirm and clear the highlight. See MIGRATION-NOTES.md.</t>
@@ -595,9 +590,9 @@
           <t>Ben</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>gtf</t>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>faculty</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Collapse the Tutor role into Learning Assistant
Most people who tutor are ENGR LAs anyway, and to a student the two
words named the same kind of help — the distinction only ever made the
Role filter longer. The four tutor-only people become `la`; their
shifts are all on the tutoring programme, so their room and course list
still resolve from `default_location_tutoring` and `courses_tutoring`
and nothing a student sees changes but the badge.

`tutor`, `peer tutor` and `tutoring` now normalize to `la` rather than
to their own role, so a workbook cell that still says "tutor" keeps
working instead of hiding the person.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/office-hours.xlsx
+++ b/data/office-hours.xlsx
@@ -1251,7 +1251,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>tutor</t>
+          <t>la</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -1268,7 +1268,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>tutor</t>
+          <t>la</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -1285,7 +1285,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>tutor</t>
+          <t>la</t>
         </is>
       </c>
     </row>
@@ -1297,7 +1297,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>tutor</t>
+          <t>la</t>
         </is>
       </c>
     </row>
@@ -1315,8 +1315,8 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="C2:C400" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not one of the choices" error="Role must be faculty, gtf, la, or tutor." type="list">
-      <formula1>"faculty,gtf,la,tutor"</formula1>
+    <dataValidation sqref="C2:C400" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not one of the choices" error="Role must be faculty, gtf, or la." type="list">
+      <formula1>"faculty,gtf,la"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5260,7 +5260,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A52"/>
+  <dimension ref="A1:A53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -5273,7 +5273,9 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
+    </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -5288,7 +5290,9 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
+    <row r="5">
+      <c r="A5" t="inlineStr"/>
+    </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
@@ -5303,7 +5307,9 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
+    <row r="8">
+      <c r="A8" t="inlineStr"/>
+    </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
@@ -5328,257 +5334,272 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  role          faculty, gtf, la, or tutor. Pick from the dropdown.</t>
+          <t xml:space="preserve">  role          faculty, gtf, or la. Pick from the dropdown.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">                Use tutor only for someone who tutors and is not also an LA.</t>
+          <t xml:space="preserve">                Everyone who tutors is an la, whether or not they also hold</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">  courses       what they help with at ENGR OFFICE HOURS.</t>
+          <t xml:space="preserve">                ENGR office hours.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">                Leave BLANK for the default (ENGR 111 and ENGR 114).</t>
+          <t xml:space="preserve">  courses       what they help with at ENGR OFFICE HOURS.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">                If you fill it in, list ALL courses they cover, separated by ;</t>
+          <t xml:space="preserve">                Leave BLANK for the default (ENGR 111 and ENGR 114).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">                Anyone covering ENGR 111 is counted for ENGR 123 too - see the</t>
+          <t xml:space="preserve">                If you fill it in, list ALL courses they cover, separated by ;</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">                course_implies row on the settings sheet.</t>
+          <t xml:space="preserve">                Anyone covering ENGR 111 is counted for ENGR 123 too - see the</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  courses_tutoring   what they can help with AT TUTORING. Separated by ;</t>
+          <t xml:space="preserve">                course_implies row on the settings sheet.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">                Blank means they do not tutor. This is the only place to edit it -</t>
+          <t xml:space="preserve">  courses_tutoring   what they can help with AT TUTORING. Separated by ;</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">                every one of their tutoring shifts reads from this cell.</t>
+          <t xml:space="preserve">                Blank means they do not tutor. This is the only place to edit it -</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t xml:space="preserve">                every one of their tutoring shifts reads from this cell.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t xml:space="preserve">  email, notes  optional. Both are shown to students, so keep notes short and useful.</t>
         </is>
       </c>
     </row>
-    <row r="23"/>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  Yellow cells were guessed during the migration - please check them.</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="5" t="inlineStr"/>
-    </row>
     <row r="26">
-      <c r="A26" s="5" t="inlineStr">
+      <c r="A26" s="5" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
         <is>
           <t>shifts sheet - one row per weekly hour</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  name          pick from the dropdown (it reads the people sheet)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">  day           Monday through Sunday. Days with no rows show as closed.</t>
+          <t xml:space="preserve">  name          pick from the dropdown (it reads the people sheet)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">  start / end   like 9:00 AM or 1:30 PM. Must land on the hour or half hour.</t>
+          <t xml:space="preserve">  day           Monday through Sunday. Days with no rows show as closed.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  program       office hours or tutoring. Blank = office hours.</t>
+          <t xml:space="preserve">  start / end   like 9:00 AM or 1:30 PM. Must land on the hour or half hour.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">                Tutoring rows take their room and their courses from tutoring:</t>
+          <t xml:space="preserve">  program       office hours or tutoring. Blank = office hours.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">                leave location and courses blank unless this one row differs.</t>
+          <t xml:space="preserve">                Tutoring rows take their room and their courses from tutoring:</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">  mode          in-person or online. Blank = in-person.</t>
+          <t xml:space="preserve">                leave location and courses blank unless this one row differs.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">  location      blank = the default room for the programme (see settings).</t>
+          <t xml:space="preserve">  mode          in-person or online. Blank = in-person.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">                Fill it in for anywhere else - Scott Engineering, etc.</t>
+          <t xml:space="preserve">  location      blank = the default room for the programme (see settings).</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">                The site gives every room its own colour automatically.</t>
+          <t xml:space="preserve">                Fill it in for anywhere else - Scott Engineering, etc.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">                For online, put the meeting link here.</t>
+          <t xml:space="preserve">                The site gives every room its own colour automatically.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">  courses       blank = whatever the people sheet says for that programme.</t>
+          <t xml:space="preserve">                For online, put the meeting link here.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
+          <t xml:space="preserve">  courses       blank = whatever the people sheet says for that programme.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
           <t xml:space="preserve">  active        put no to hide a row for a while without deleting it.</t>
         </is>
       </c>
     </row>
-    <row r="40"/>
     <row r="41">
-      <c r="A41" s="5" t="inlineStr">
+      <c r="A41" s="5" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
         <is>
           <t>exceptions sheet - one-off changes to the normal week</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Cancel one shift:  name, date, start, end, type = cancelled</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Cancel a whole day for someone: leave start and end blank</t>
+          <t xml:space="preserve">  Cancel one shift:  name, date, start, end, type = cancelled</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Cancel a whole day for someone: leave start and end blank</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Add extra hours:   name, date, start, end, type = added</t>
         </is>
       </c>
     </row>
-    <row r="45"/>
     <row r="46">
-      <c r="A46" s="5" t="inlineStr">
+      <c r="A46" s="5" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
         <is>
           <t>settings sheet - term dates, default rooms, and the announcement banner</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  default_location_tutoring   the tutoring room. One edit moves the whole</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">                              programme.</t>
+          <t xml:space="preserve">  default_location_tutoring   the tutoring room. One edit moves the whole</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">  subjects                    groups the courses in the Get help with menu.</t>
+          <t xml:space="preserve">                              programme.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
+          <t xml:space="preserve">  subjects                    groups the courses in the Get help with menu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
           <t xml:space="preserve">  course_order                the order that menu lists them in.</t>
         </is>
       </c>
     </row>
-    <row r="51"/>
     <row r="52">
-      <c r="A52" t="inlineStr">
+      <c r="A52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
         <is>
           <t>When you are done: save, then send the file to Ben (or save it back to OneDrive).</t>
         </is>

</xml_diff>

<commit_message>
Give languages a column and a filter of their own
The rota's "Bilingual Tutors!" note was already being read, but it
landed in `people.notes` as "Also tutors in Spanish." — prose nobody
could filter on, written into a cell a human might have typed in.

It gets `people.languages` instead: a `;` list of languages besides
English, which fills a new Language filter and an "Also speaks" line in
the panel. English is never an option, since everyone here speaks it
and offering it would filter nothing out.

Language belongs to the person, not the shift, so it applies at office
hours as much as at tutoring — filtering to Hungarian finds Tia
Fountain's Thursday hour in C144 as well as her tutoring in C141.
add_tutoring.py rebuilds the column every run, blanking anyone dropped
from the bilingual list.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/office-hours.xlsx
+++ b/data/office-hours.xlsx
@@ -511,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G50"/>
+  <dimension ref="A1:H50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -521,6 +521,7 @@
     <col width="26" customWidth="1" min="5" max="5"/>
     <col width="46" customWidth="1" min="6" max="6"/>
     <col width="44" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -559,6 +560,11 @@
           <t>courses_tutoring</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>languages</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -571,14 +577,14 @@
           <t>la</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Also tutors in Spanish.</t>
-        </is>
-      </c>
       <c r="G2" t="inlineStr">
         <is>
           <t>CHEM 111; CHEM 112; CHEM 113; CHEM 114; CHEM 120; CHEM 121; PH 141; Precalculus; MATH 160; MATH 161; MATH 261; MATH 340</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Spanish</t>
         </is>
       </c>
     </row>
@@ -762,14 +768,14 @@
           <t>la</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Also tutors in Spanish.</t>
-        </is>
-      </c>
       <c r="G15" t="inlineStr">
         <is>
           <t>PH 141; MATH 160; MATH 161</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Spanish</t>
         </is>
       </c>
     </row>
@@ -1060,14 +1066,14 @@
           <t>la</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>Also tutors in Bengali.</t>
-        </is>
-      </c>
       <c r="G34" t="inlineStr">
         <is>
           <t>PH 141; PH 142; Precalculus; MATH 160; MATH 161; ENGR 111; ENGR 114</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Bengali</t>
         </is>
       </c>
     </row>
@@ -1099,14 +1105,14 @@
           <t>la</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>Also tutors in Spanish.</t>
-        </is>
-      </c>
       <c r="G36" t="inlineStr">
         <is>
           <t>CHEM 111; CHEM 112; CHEM 113; CHEM 114; PH 141; Precalculus; MATH 160; MATH 161; MATH 261; MATH 340; CIVE 261; CIVE 360; CIVE 260; ENGR 111; ENGR 114</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Spanish</t>
         </is>
       </c>
     </row>
@@ -1191,14 +1197,14 @@
           <t>la</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>Also tutors in Hungarian.</t>
-        </is>
-      </c>
       <c r="G42" t="inlineStr">
         <is>
           <t>CHEM 120; CHEM 121; CHEM 341; PH 141; Precalculus; MATH 160</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Hungarian</t>
         </is>
       </c>
     </row>
@@ -5260,7 +5266,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A53"/>
+  <dimension ref="A1:A56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -5273,9 +5279,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -5290,9 +5294,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr"/>
-    </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
@@ -5307,9 +5309,7 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr"/>
-    </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
@@ -5411,195 +5411,208 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">  email, notes  optional. Both are shown to students, so keep notes short and useful.</t>
+          <t xml:space="preserve">  languages     languages BESIDES ENGLISH they can help in, separated by ;</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr"/>
+      <c r="A24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                Blank for most people. Becomes the Language filter and a</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Yellow cells were guessed during the migration - please check them.</t>
+          <t xml:space="preserve">                line in the panel. Rebuilt from the rota's bilingual list.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="inlineStr"/>
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  email, notes  optional. Both are shown to students, so keep notes short and useful.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="5" t="inlineStr">
-        <is>
-          <t>shifts sheet - one row per weekly hour</t>
-        </is>
-      </c>
+      <c r="A27" s="5" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">  name          pick from the dropdown (it reads the people sheet)</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  day           Monday through Sunday. Days with no rows show as closed.</t>
-        </is>
-      </c>
-    </row>
+          <t xml:space="preserve">  Yellow cells were guessed during the migration - please check them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29"/>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  start / end   like 9:00 AM or 1:30 PM. Must land on the hour or half hour.</t>
+          <t>shifts sheet - one row per weekly hour</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  program       office hours or tutoring. Blank = office hours.</t>
+          <t xml:space="preserve">  name          pick from the dropdown (it reads the people sheet)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">                Tutoring rows take their room and their courses from tutoring:</t>
+          <t xml:space="preserve">  day           Monday through Sunday. Days with no rows show as closed.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">                leave location and courses blank unless this one row differs.</t>
+          <t xml:space="preserve">  start / end   like 9:00 AM or 1:30 PM. Must land on the hour or half hour.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">  mode          in-person or online. Blank = in-person.</t>
+          <t xml:space="preserve">  program       office hours or tutoring. Blank = office hours.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">  location      blank = the default room for the programme (see settings).</t>
+          <t xml:space="preserve">                Tutoring rows take their room and their courses from tutoring:</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">                Fill it in for anywhere else - Scott Engineering, etc.</t>
+          <t xml:space="preserve">                leave location and courses blank unless this one row differs.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">                The site gives every room its own colour automatically.</t>
+          <t xml:space="preserve">  mode          in-person or online. Blank = in-person.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">                For online, put the meeting link here.</t>
+          <t xml:space="preserve">  location      blank = the default room for the programme (see settings).</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">  courses       blank = whatever the people sheet says for that programme.</t>
+          <t xml:space="preserve">                Fill it in for anywhere else - Scott Engineering, etc.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">  active        put no to hide a row for a while without deleting it.</t>
+          <t xml:space="preserve">                The site gives every room its own colour automatically.</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="5" t="inlineStr"/>
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                For online, put the meeting link here.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>exceptions sheet - one-off changes to the normal week</t>
+          <t xml:space="preserve">  courses       blank = whatever the people sheet says for that programme.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
+          <t xml:space="preserve">  active        put no to hide a row for a while without deleting it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44"/>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>exceptions sheet - one-off changes to the normal week</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Cancel one shift:  name, date, start, end, type = cancelled</t>
         </is>
       </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Cancel a whole day for someone: leave start and end blank</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Add extra hours:   name, date, start, end, type = added</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="5" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>settings sheet - term dates, default rooms, and the announcement banner</t>
+          <t xml:space="preserve">  Cancel a whole day for someone: leave start and end blank</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">  default_location_tutoring   the tutoring room. One edit moves the whole</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">                              programme.</t>
-        </is>
-      </c>
-    </row>
+          <t xml:space="preserve">  Add extra hours:   name, date, start, end, type = added</t>
+        </is>
+      </c>
+    </row>
+    <row r="49"/>
     <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  subjects                    groups the courses in the Get help with menu.</t>
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>settings sheet - term dates, default rooms, and the announcement banner</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t xml:space="preserve">  course_order                the order that menu lists them in.</t>
+          <t xml:space="preserve">  default_location_tutoring   the tutoring room. One edit moves the whole</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr"/>
+      <c r="A52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                              programme.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  subjects                    groups the courses in the Get help with menu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  course_order                the order that menu lists them in.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55"/>
+    <row r="56">
+      <c r="A56" t="inlineStr">
         <is>
           <t>When you are done: save, then send the file to Ben (or save it back to OneDrive).</t>
         </is>

</xml_diff>

<commit_message>
Fold the updated Faculty & GTF grid into the workbook
One change on the grid: Winnie's Wednesday 12-1 PM hour moves to Friday
9-10 AM. Dr. Dan keeps the Wednesday hour on his own. Everything else,
and everyone else, is unchanged.

Applied with update_faculty_hours.py, whose diff matched a cell-by-cell
comparison of the two grids exactly. The tutoring rota and the LA grid
that arrived alongside it were both identical to the copies already in
source-data, so neither moved anything.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/office-hours.xlsx
+++ b/data/office-hours.xlsx
@@ -2196,7 +2196,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Winnie</t>
+          <t>Dr. Yume</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2206,19 +2206,19 @@
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>12:00 PM</t>
+          <t>1:00 PM</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>1:00 PM</t>
+          <t>2:00 PM</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Dr. Yume</t>
+          <t>River Wysock</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2240,7 +2240,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>River Wysock</t>
+          <t>DrT</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2250,19 +2250,19 @@
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>1:00 PM</t>
+          <t>2:00 PM</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>2:00 PM</t>
+          <t>3:00 PM</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>DrT</t>
+          <t>Joseph Quiroz Hernandez</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2284,7 +2284,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Joseph Quiroz Hernandez</t>
+          <t>DrT</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2294,19 +2294,19 @@
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>2:00 PM</t>
+          <t>3:00 PM</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>3:00 PM</t>
+          <t>4:00 PM</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>DrT</t>
+          <t>Hannah Gruber</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2328,7 +2328,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Hannah Gruber</t>
+          <t>Sumaiya</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2338,41 +2338,41 @@
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>3:00 PM</t>
+          <t>5:00 PM</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>4:00 PM</t>
+          <t>6:00 PM</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Sumaiya</t>
+          <t>Sylvia Ingegneri</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>5:00 PM</t>
+          <t>9:00 AM</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>6:00 PM</t>
+          <t>10:00 AM</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Sylvia Ingegneri</t>
+          <t>Parker Bjick</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2382,19 +2382,19 @@
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>9:00 AM</t>
+          <t>10:00 AM</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>10:00 AM</t>
+          <t>11:00 AM</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Parker Bjick</t>
+          <t>Taylor</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2416,7 +2416,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Taylor</t>
+          <t>Austin Monroe</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2426,19 +2426,19 @@
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>10:00 AM</t>
+          <t>11:00 AM</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>11:00 AM</t>
+          <t>12:00 PM</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Austin Monroe</t>
+          <t>Taylor</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2460,7 +2460,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Taylor</t>
+          <t>Ojo</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2470,19 +2470,19 @@
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>11:00 AM</t>
+          <t>12:00 PM</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>12:00 PM</t>
+          <t>1:00 PM</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Ojo</t>
+          <t>Tia Fountain</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2504,7 +2504,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Tia Fountain</t>
+          <t>Dr. Harvey</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2514,19 +2514,19 @@
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>12:00 PM</t>
+          <t>1:00 PM</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>1:00 PM</t>
+          <t>2:00 PM</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Dr. Harvey</t>
+          <t>Sarah Goudjil</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2548,7 +2548,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Sarah Goudjil</t>
+          <t>Dr. Harvey</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2558,19 +2558,19 @@
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>1:00 PM</t>
+          <t>2:00 PM</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>2:00 PM</t>
+          <t>3:00 PM</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Dr. Harvey</t>
+          <t>Prof Scheller</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2592,7 +2592,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Prof Scheller</t>
+          <t>Tucker Cullen</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2608,13 +2608,23 @@
       <c r="D55" s="4" t="inlineStr">
         <is>
           <t>3:00 PM</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>online</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>https://teams.microsoft.com/l/message/19:42625ed077084999881c0275e689deec@thread.v2/1787625651798?context=%7B%22contextType%22%3A%22chat%22%7D</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Tucker Cullen</t>
+          <t>Julie Rickerd</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2624,29 +2634,19 @@
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>2:00 PM</t>
+          <t>3:00 PM</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>3:00 PM</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>online</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>https://teams.microsoft.com/l/message/19:42625ed077084999881c0275e689deec@thread.v2/1787625651798?context=%7B%22contextType%22%3A%22chat%22%7D</t>
+          <t>4:00 PM</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Julie Rickerd</t>
+          <t>Prof Scheller</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2668,7 +2668,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Prof Scheller</t>
+          <t>Ojo</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2678,12 +2678,12 @@
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>3:00 PM</t>
+          <t>4:00 PM</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t>4:00 PM</t>
+          <t>5:00 PM</t>
         </is>
       </c>
     </row>
@@ -2700,41 +2700,41 @@
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>4:00 PM</t>
+          <t>5:00 PM</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t>5:00 PM</t>
+          <t>6:00 PM</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Ojo</t>
+          <t>Thomas Miller</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>5:00 PM</t>
+          <t>9:00 AM</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t>6:00 PM</t>
+          <t>10:00 AM</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Thomas Miller</t>
+          <t>Winnie</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -5279,7 +5279,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -5294,7 +5293,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
@@ -5309,7 +5307,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
@@ -5446,7 +5443,6 @@
         </is>
       </c>
     </row>
-    <row r="29"/>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
@@ -5545,7 +5541,6 @@
         </is>
       </c>
     </row>
-    <row r="44"/>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
@@ -5574,7 +5569,6 @@
         </is>
       </c>
     </row>
-    <row r="49"/>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
@@ -5610,7 +5604,6 @@
         </is>
       </c>
     </row>
-    <row r="55"/>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Move Prof Scheller's three hours off Tuesday and Thursday
Their Tuesday 2-3, Thursday 2-3 and Thursday 3-4 shifts in AV C144 are
now Monday 11-12, Wednesday 4-5 and Thursday 2:30-3:30. Room, name and
the rest of the sheet are unchanged; no other person's hours moved.

The three cells were re-entered as Excel time values (h:mm AM/PM)
rather than the "2:00 PM" text the other rows use. That reads the same
in the browser - xlsx.js hands parseTime the day fraction and it takes
the numeric path - so the display is unaffected.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/office-hours.xlsx
+++ b/data/office-hours.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bengrier/Desktop/CSU Work/AI App Creation/Office Hours Display/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB0CF16D-2290-AC42-9B68-DC201CA51327}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DAEDD2F-EB34-5B40-B182-65870971DB08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-32020" yWindow="-3960" windowWidth="30240" windowHeight="18880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="people" sheetId="1" r:id="rId1"/>
@@ -195,7 +195,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="942" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="936" uniqueCount="200">
   <si>
     <t>name</t>
   </si>
@@ -853,7 +853,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -864,6 +864,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="18" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1697,7 +1698,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <sheetPr>
+  <sheetPr filterMode="1">
     <tabColor rgb="FF1F3864"/>
   </sheetPr>
   <dimension ref="A1:E142"/>
@@ -1726,7 +1727,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>20</v>
       </c>
@@ -1743,7 +1744,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>40</v>
       </c>
@@ -1760,7 +1761,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>57</v>
       </c>
@@ -1777,7 +1778,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -1794,7 +1795,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>42</v>
       </c>
@@ -1811,7 +1812,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -1828,7 +1829,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>18</v>
       </c>
@@ -1845,7 +1846,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>34</v>
       </c>
@@ -1862,7 +1863,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>84</v>
       </c>
@@ -1879,7 +1880,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -1896,7 +1897,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>26</v>
       </c>
@@ -1913,7 +1914,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>84</v>
       </c>
@@ -1930,7 +1931,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>57</v>
       </c>
@@ -1947,7 +1948,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>62</v>
       </c>
@@ -1964,7 +1965,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>26</v>
       </c>
@@ -1981,7 +1982,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>30</v>
       </c>
@@ -1998,7 +1999,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>36</v>
       </c>
@@ -2015,7 +2016,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>65</v>
       </c>
@@ -2032,7 +2033,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>24</v>
       </c>
@@ -2049,7 +2050,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>26</v>
       </c>
@@ -2066,7 +2067,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>43</v>
       </c>
@@ -2083,7 +2084,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>65</v>
       </c>
@@ -2100,7 +2101,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>24</v>
       </c>
@@ -2117,7 +2118,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>38</v>
       </c>
@@ -2134,7 +2135,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>57</v>
       </c>
@@ -2151,7 +2152,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>4</v>
       </c>
@@ -2168,7 +2169,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>24</v>
       </c>
@@ -2185,7 +2186,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>38</v>
       </c>
@@ -2202,7 +2203,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>40</v>
       </c>
@@ -2219,7 +2220,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>4</v>
       </c>
@@ -2236,7 +2237,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>80</v>
       </c>
@@ -2253,7 +2254,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>40</v>
       </c>
@@ -2270,7 +2271,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>4</v>
       </c>
@@ -2287,7 +2288,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>68</v>
       </c>
@@ -2304,7 +2305,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>43</v>
       </c>
@@ -2321,7 +2322,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>23</v>
       </c>
@@ -2338,7 +2339,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>84</v>
       </c>
@@ -2355,7 +2356,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>19</v>
       </c>
@@ -2372,7 +2373,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>30</v>
       </c>
@@ -2389,7 +2390,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>19</v>
       </c>
@@ -2406,7 +2407,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>45</v>
       </c>
@@ -2428,19 +2429,19 @@
         <v>55</v>
       </c>
       <c r="B43" t="s">
-        <v>105</v>
-      </c>
-      <c r="C43" t="s">
-        <v>95</v>
-      </c>
-      <c r="D43" t="s">
-        <v>96</v>
+        <v>89</v>
+      </c>
+      <c r="C43" s="6">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="D43" s="6">
+        <v>0.5</v>
       </c>
       <c r="E43" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>10</v>
       </c>
@@ -2457,7 +2458,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>15</v>
       </c>
@@ -2474,7 +2475,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>45</v>
       </c>
@@ -2491,7 +2492,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>64</v>
       </c>
@@ -2508,7 +2509,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>69</v>
       </c>
@@ -2525,7 +2526,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>10</v>
       </c>
@@ -2542,7 +2543,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>11</v>
       </c>
@@ -2559,7 +2560,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>15</v>
       </c>
@@ -2576,7 +2577,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>21</v>
       </c>
@@ -2593,7 +2594,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>45</v>
       </c>
@@ -2610,7 +2611,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>10</v>
       </c>
@@ -2627,7 +2628,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>11</v>
       </c>
@@ -2644,7 +2645,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>21</v>
       </c>
@@ -2661,7 +2662,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>60</v>
       </c>
@@ -2678,7 +2679,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>78</v>
       </c>
@@ -2695,7 +2696,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>60</v>
       </c>
@@ -2712,7 +2713,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>66</v>
       </c>
@@ -2729,7 +2730,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>13</v>
       </c>
@@ -2746,7 +2747,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>78</v>
       </c>
@@ -2763,7 +2764,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>60</v>
       </c>
@@ -2780,7 +2781,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>66</v>
       </c>
@@ -2797,7 +2798,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>13</v>
       </c>
@@ -2814,7 +2815,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>60</v>
       </c>
@@ -2831,7 +2832,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>26</v>
       </c>
@@ -2848,7 +2849,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>15</v>
       </c>
@@ -2865,7 +2866,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>51</v>
       </c>
@@ -2882,7 +2883,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>11</v>
       </c>
@@ -2899,7 +2900,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>33</v>
       </c>
@@ -2916,7 +2917,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>17</v>
       </c>
@@ -2933,7 +2934,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>38</v>
       </c>
@@ -2950,7 +2951,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>19</v>
       </c>
@@ -2967,7 +2968,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>56</v>
       </c>
@@ -2984,7 +2985,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>20</v>
       </c>
@@ -3001,7 +3002,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>28</v>
       </c>
@@ -3018,7 +3019,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>8</v>
       </c>
@@ -3035,7 +3036,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>20</v>
       </c>
@@ -3052,7 +3053,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>21</v>
       </c>
@@ -3069,7 +3070,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>28</v>
       </c>
@@ -3086,7 +3087,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>40</v>
       </c>
@@ -3103,7 +3104,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>28</v>
       </c>
@@ -3120,7 +3121,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>30</v>
       </c>
@@ -3137,7 +3138,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>51</v>
       </c>
@@ -3154,7 +3155,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>71</v>
       </c>
@@ -3171,7 +3172,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>57</v>
       </c>
@@ -3188,7 +3189,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>62</v>
       </c>
@@ -3205,7 +3206,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>65</v>
       </c>
@@ -3222,7 +3223,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>71</v>
       </c>
@@ -3239,7 +3240,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>62</v>
       </c>
@@ -3256,7 +3257,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>66</v>
       </c>
@@ -3273,7 +3274,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>60</v>
       </c>
@@ -3290,7 +3291,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
         <v>62</v>
       </c>
@@ -3307,7 +3308,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>80</v>
       </c>
@@ -3324,7 +3325,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>62</v>
       </c>
@@ -3341,7 +3342,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>66</v>
       </c>
@@ -3358,7 +3359,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>53</v>
       </c>
@@ -3375,7 +3376,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>68</v>
       </c>
@@ -3392,7 +3393,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>10</v>
       </c>
@@ -3409,7 +3410,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
         <v>68</v>
       </c>
@@ -3426,7 +3427,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
         <v>49</v>
       </c>
@@ -3443,7 +3444,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
         <v>71</v>
       </c>
@@ -3460,7 +3461,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
         <v>18</v>
       </c>
@@ -3477,7 +3478,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
         <v>60</v>
       </c>
@@ -3494,7 +3495,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
         <v>18</v>
       </c>
@@ -3516,19 +3517,19 @@
         <v>55</v>
       </c>
       <c r="B107" t="s">
-        <v>109</v>
-      </c>
-      <c r="C107" t="s">
-        <v>95</v>
-      </c>
-      <c r="D107" t="s">
-        <v>96</v>
+        <v>107</v>
+      </c>
+      <c r="C107" s="6">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="D107" s="6">
+        <v>0.70833333333333337</v>
       </c>
       <c r="E107" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
         <v>75</v>
       </c>
@@ -3545,7 +3546,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
         <v>32</v>
       </c>
@@ -3562,7 +3563,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
         <v>36</v>
       </c>
@@ -3579,7 +3580,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
         <v>38</v>
       </c>
@@ -3603,17 +3604,17 @@
       <c r="B112" t="s">
         <v>109</v>
       </c>
-      <c r="C112" t="s">
-        <v>96</v>
-      </c>
-      <c r="D112" t="s">
-        <v>97</v>
+      <c r="C112" s="6">
+        <v>0.60416666666666663</v>
+      </c>
+      <c r="D112" s="6">
+        <v>0.64583333333333337</v>
       </c>
       <c r="E112" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
         <v>69</v>
       </c>
@@ -3630,7 +3631,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
         <v>38</v>
       </c>
@@ -3647,7 +3648,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
         <v>49</v>
       </c>
@@ -3664,7 +3665,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
         <v>75</v>
       </c>
@@ -3681,7 +3682,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
         <v>78</v>
       </c>
@@ -3698,7 +3699,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
         <v>78</v>
       </c>
@@ -3715,7 +3716,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
         <v>34</v>
       </c>
@@ -3732,7 +3733,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
         <v>49</v>
       </c>
@@ -3749,7 +3750,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
         <v>78</v>
       </c>
@@ -3766,7 +3767,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
         <v>34</v>
       </c>
@@ -3783,7 +3784,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
         <v>75</v>
       </c>
@@ -3800,7 +3801,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
         <v>80</v>
       </c>
@@ -3817,7 +3818,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
         <v>34</v>
       </c>
@@ -3834,7 +3835,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
         <v>47</v>
       </c>
@@ -3851,7 +3852,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
         <v>75</v>
       </c>
@@ -3868,7 +3869,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
         <v>80</v>
       </c>
@@ -3885,7 +3886,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
         <v>47</v>
       </c>
@@ -3902,7 +3903,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A130" t="s">
         <v>69</v>
       </c>
@@ -3919,7 +3920,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A131" t="s">
         <v>77</v>
       </c>
@@ -3936,7 +3937,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A132" t="s">
         <v>47</v>
       </c>
@@ -3953,7 +3954,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A133" t="s">
         <v>77</v>
       </c>
@@ -3970,7 +3971,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A134" t="s">
         <v>24</v>
       </c>
@@ -3987,7 +3988,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A135" t="s">
         <v>13</v>
       </c>
@@ -4004,7 +4005,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A136" t="s">
         <v>77</v>
       </c>
@@ -4021,7 +4022,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A137" t="s">
         <v>36</v>
       </c>
@@ -4038,7 +4039,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A138" t="s">
         <v>50</v>
       </c>
@@ -4055,7 +4056,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A139" t="s">
         <v>74</v>
       </c>
@@ -4072,7 +4073,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A140" t="s">
         <v>56</v>
       </c>
@@ -4089,7 +4090,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A141" t="s">
         <v>56</v>
       </c>
@@ -4106,7 +4107,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A142" t="s">
         <v>56</v>
       </c>
@@ -4124,7 +4125,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E142" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A1:E142" xr:uid="{00000000-0009-0000-0000-000001000000}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="Prof Scheller"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Check this cell" error="Pick a name from the people sheet. Add them there first if they are new." sqref="A2:A341" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>PeopleNames</formula1>

</xml_diff>